<commit_message>
Add graph color palette and enhance chart styling in grafici.html
</commit_message>
<xml_diff>
--- a/Utenze_main.xlsx
+++ b/Utenze_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camozzicloud-my.sharepoint.com/personal/mpasseri_fonderiemoragavardo_it/Documents/Documenti/VSCode/EnergyMeters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="282" documentId="11_CD3F85A73935972BAC2112A087E31DD0A106565D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A330F1BB-50A7-4A6E-88F8-F9091A6645AE}"/>
+  <xr:revisionPtr revIDLastSave="284" documentId="11_CD3F85A73935972BAC2112A087E31DD0A106565D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBF1C138-31A9-480B-AF6A-7B2912005102}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -155,9 +155,6 @@
     <t>Compressore Rn160e Nirvana</t>
   </si>
   <si>
-    <t>Comressore Compair L200</t>
-  </si>
-  <si>
     <t>Utenze varie formatura mano</t>
   </si>
   <si>
@@ -180,6 +177,9 @@
   </si>
   <si>
     <t>Filtro E35 Gostol/Lamef</t>
+  </si>
+  <si>
+    <t>Compressore Compair L200 (Blastman)</t>
   </si>
 </sst>
 </file>
@@ -907,7 +907,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -964,7 +964,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -978,7 +978,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31">
         <v>2</v>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B33">
         <v>2</v>
@@ -1020,7 +1020,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B34">
         <v>2</v>
@@ -1029,7 +1029,7 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1140,7 +1140,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B44">
         <v>2</v>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B53">
         <v>3</v>
@@ -1277,7 +1277,7 @@
         <v>5</v>
       </c>
       <c r="D54" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -1363,7 +1363,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B62">
         <v>3</v>

</xml_diff>

<commit_message>
Update Utenze_main.xlsx binary file
</commit_message>
<xml_diff>
--- a/Utenze_main.xlsx
+++ b/Utenze_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camozzicloud-my.sharepoint.com/personal/mpasseri_fonderiemoragavardo_it/Documents/Documenti/VSCode/EnergyMeters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="295" documentId="11_CD3F85A73935972BAC2112A087E31DD0A106565D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49461C87-F1B3-4D2E-AD80-50F67F395736}"/>
+  <xr:revisionPtr revIDLastSave="339" documentId="11_CD3F85A73935972BAC2112A087E31DD0A106565D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{970CC885-4EEB-4972-A860-8EFA795FE888}"/>
   <bookViews>
-    <workbookView xWindow="30645" yWindow="2730" windowWidth="21600" windowHeight="11175" tabRatio="140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="51">
   <si>
     <t>Cabinet</t>
   </si>
@@ -50,9 +50,6 @@
     <t>CAB1 GEN2</t>
   </si>
   <si>
-    <t>Group</t>
-  </si>
-  <si>
     <t>Generali</t>
   </si>
   <si>
@@ -183,13 +180,19 @@
   </si>
   <si>
     <t>Quadro luci cabina 1</t>
+  </si>
+  <si>
+    <t>Group1</t>
+  </si>
+  <si>
+    <t>Group2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -201,6 +204,12 @@
       <u/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -572,15 +581,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.58203125" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.08203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -591,24 +601,30 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3">
         <v>1</v>
       </c>
@@ -616,12 +632,15 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -630,12 +649,15 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -644,12 +666,15 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -658,12 +683,15 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -672,12 +700,15 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -686,12 +717,15 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -700,10 +734,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>1</v>
       </c>
@@ -711,10 +748,13 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>1</v>
       </c>
@@ -722,12 +762,15 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -736,12 +779,15 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -750,10 +796,13 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -764,12 +813,15 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -778,10 +830,13 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16">
         <v>1</v>
@@ -790,13 +845,16 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E16" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -805,12 +863,15 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -819,10 +880,13 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>1</v>
       </c>
@@ -830,12 +894,15 @@
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -844,12 +911,15 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -858,10 +928,13 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B22">
         <v>1</v>
       </c>
@@ -869,12 +942,15 @@
         <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -883,12 +959,15 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -897,10 +976,13 @@
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>1</v>
       </c>
@@ -908,12 +990,15 @@
         <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -922,12 +1007,15 @@
         <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -936,13 +1024,16 @@
         <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -951,12 +1042,15 @@
         <v>27</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B29">
         <v>2</v>
@@ -967,10 +1061,13 @@
       <c r="D29" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E29" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -979,12 +1076,15 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B31">
         <v>2</v>
@@ -993,12 +1093,15 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32">
         <v>2</v>
@@ -1007,12 +1110,15 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B33">
         <v>2</v>
@@ -1021,12 +1127,15 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E33" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B34">
         <v>2</v>
@@ -1035,12 +1144,15 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35">
         <v>2</v>
@@ -1049,10 +1161,13 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E35" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>2</v>
       </c>
@@ -1060,10 +1175,13 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B37">
         <v>2</v>
       </c>
@@ -1071,10 +1189,13 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B38">
         <v>2</v>
       </c>
@@ -1082,10 +1203,13 @@
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B39">
         <v>2</v>
       </c>
@@ -1093,10 +1217,13 @@
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B40">
         <v>2</v>
       </c>
@@ -1104,10 +1231,13 @@
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B41">
         <v>2</v>
       </c>
@@ -1115,12 +1245,15 @@
         <v>13</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -1129,10 +1262,13 @@
         <v>14</v>
       </c>
       <c r="D42" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
       <c r="B43">
         <v>2</v>
@@ -1141,12 +1277,15 @@
         <v>15</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B44">
         <v>2</v>
@@ -1155,12 +1294,15 @@
         <v>16</v>
       </c>
       <c r="D44" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E44" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B45">
         <v>2</v>
@@ -1169,10 +1311,13 @@
         <v>17</v>
       </c>
       <c r="D45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B46">
         <v>2</v>
       </c>
@@ -1180,12 +1325,15 @@
         <v>18</v>
       </c>
       <c r="D46" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B47">
         <v>2</v>
@@ -1194,10 +1342,13 @@
         <v>19</v>
       </c>
       <c r="D47" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E47" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B48">
         <v>2</v>
       </c>
@@ -1205,10 +1356,13 @@
         <v>20</v>
       </c>
       <c r="D48" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E48" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B49">
         <v>2</v>
       </c>
@@ -1216,38 +1370,47 @@
         <v>21</v>
       </c>
       <c r="D49" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="E49" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
+        <v>10</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s">
         <v>11</v>
       </c>
-      <c r="B50">
-        <v>3</v>
-      </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>46</v>
-      </c>
-      <c r="B51">
-        <v>3</v>
-      </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B52">
         <v>3</v>
       </c>
@@ -1255,12 +1418,15 @@
         <v>3</v>
       </c>
       <c r="D52" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B53">
         <v>3</v>
@@ -1269,12 +1435,15 @@
         <v>4</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B54">
         <v>3</v>
@@ -1283,12 +1452,15 @@
         <v>5</v>
       </c>
       <c r="D54" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E54" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B55">
         <v>3</v>
@@ -1297,10 +1469,13 @@
         <v>6</v>
       </c>
       <c r="D55" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B56">
         <v>3</v>
       </c>
@@ -1308,10 +1483,13 @@
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B57">
         <v>3</v>
       </c>
@@ -1319,10 +1497,13 @@
         <v>8</v>
       </c>
       <c r="D57" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B58">
         <v>3</v>
       </c>
@@ -1330,10 +1511,13 @@
         <v>9</v>
       </c>
       <c r="D58" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E58" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B59">
         <v>3</v>
       </c>
@@ -1341,10 +1525,13 @@
         <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E59" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B60">
         <v>3</v>
       </c>
@@ -1352,11 +1539,14 @@
         <v>11</v>
       </c>
       <c r="D60" t="s">
-        <v>25</v>
-      </c>
-      <c r="F60" s="1"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E60" t="s">
+        <v>24</v>
+      </c>
+      <c r="G60" s="1"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B61">
         <v>3</v>
       </c>
@@ -1364,12 +1554,15 @@
         <v>12</v>
       </c>
       <c r="D61" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E61" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B62">
         <v>3</v>
@@ -1378,12 +1571,15 @@
         <v>13</v>
       </c>
       <c r="D62" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E62" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B63">
         <v>3</v>
@@ -1392,12 +1588,15 @@
         <v>14</v>
       </c>
       <c r="D63" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E63" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B64">
         <v>3</v>
@@ -1406,12 +1605,15 @@
         <v>15</v>
       </c>
       <c r="D64" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="E64" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B65">
         <v>3</v>
@@ -1420,10 +1622,14 @@
         <v>16</v>
       </c>
       <c r="D65" t="s">
-        <v>26</v>
+        <v>10</v>
+      </c>
+      <c r="E65" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>